<commit_message>
Updates for adding the variants were added
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2075072A-2960-4209-9F00-FA52B58C4930}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD620C1E-1553-40FA-A279-74702F5A5A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="111">
   <si>
     <t>Name</t>
   </si>
@@ -373,16 +373,32 @@
   <si>
     <t>El rango por defecto</t>
   </si>
+  <si>
+    <t>LayOutSAP</t>
+  </si>
+  <si>
+    <t>/ROCKETBOT</t>
+  </si>
+  <si>
+    <t>Nombre del layout para las transacciones SAP</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="17" x14ac:knownFonts="1">
+  <fonts count="18" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -513,27 +529,28 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -924,7 +941,17 @@
         <v>107</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="18" t="s">
+        <v>108</v>
+      </c>
+      <c r="B14" s="18" t="s">
+        <v>109</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>110</v>
+      </c>
+    </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
New version to try to reduce de long time in the COHV transaction was published
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD620C1E-1553-40FA-A279-74702F5A5A1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDA1352-43BE-4179-B15E-1E2E0669C0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -94,9 +94,6 @@
     <t>ExScreenshotsFolderPath</t>
   </si>
   <si>
-    <t>Exceptions_Screenshots</t>
-  </si>
-  <si>
     <t>Where to save exceptions screenshots - can be a full or a relative path.</t>
   </si>
   <si>
@@ -381,6 +378,9 @@
   </si>
   <si>
     <t>Nombre del layout para las transacciones SAP</t>
+  </si>
+  <si>
+    <t>C:\Users\aci-cns\Documents\Test UiPath\Informe seguimiento Repuestos\Exceptions_Screenshots</t>
   </si>
 </sst>
 </file>
@@ -836,7 +836,7 @@
         <v>9</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C4" s="2" t="s">
         <v>10</v>
@@ -844,13 +844,13 @@
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>55</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -866,90 +866,90 @@
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B7" s="8" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B8" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="5" t="s">
         <v>76</v>
-      </c>
-      <c r="B8" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="5" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
+        <v>89</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>88</v>
+      </c>
+      <c r="C10" s="5" t="s">
         <v>90</v>
-      </c>
-      <c r="B10" s="10" t="s">
-        <v>89</v>
-      </c>
-      <c r="C10" s="5" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="14" t="s">
+        <v>97</v>
+      </c>
+      <c r="B11" s="14" t="s">
         <v>98</v>
       </c>
-      <c r="B11" s="14" t="s">
-        <v>99</v>
-      </c>
       <c r="C11" s="5" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B12" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="B12" s="17" t="s">
-        <v>103</v>
-      </c>
       <c r="C12" s="5" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="16" t="s">
+        <v>103</v>
+      </c>
+      <c r="B13" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="B13" s="16" t="s">
-        <v>105</v>
-      </c>
       <c r="C13" s="5" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="18" t="s">
+        <v>107</v>
+      </c>
+      <c r="B14" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="C14" s="5" t="s">
         <v>109</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>110</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2013,109 +2013,109 @@
         <v>17</v>
       </c>
       <c r="B4" s="3" t="s">
+        <v>110</v>
+      </c>
+      <c r="C4" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="C4" s="3" t="s">
-        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="B5" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="C5" s="3" t="s">
         <v>21</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
+        <v>22</v>
+      </c>
+      <c r="B6" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="C6" s="3" t="s">
         <v>24</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>25</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B7" s="3" t="s">
         <v>26</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="C7" s="3" t="s">
         <v>27</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B8" s="3" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="C8" s="3" t="s">
         <v>30</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="B9" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="C9" s="3" t="s">
         <v>33</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3" t="s">
+        <v>34</v>
+      </c>
+      <c r="B10" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="C10" s="3" t="s">
         <v>36</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B11" s="3">
         <v>2</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B12" s="3">
         <v>2</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>42</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
@@ -3126,13 +3126,13 @@
         <v>0</v>
       </c>
       <c r="B1" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="C1" s="11" t="s">
         <v>44</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="D1" s="11" t="s">
         <v>45</v>
-      </c>
-      <c r="D1" s="11" t="s">
-        <v>46</v>
       </c>
       <c r="E1" s="11"/>
       <c r="F1" s="11"/>
@@ -3159,212 +3159,212 @@
     </row>
     <row r="2" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B2" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C2" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D2" s="10" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="3" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="7" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="8" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="10" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="13" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C10" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C11" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B12" s="12" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B13" s="12" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B14" s="12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D14" s="12" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B15" s="12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C15" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="B16" s="15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>7</v>
       </c>
       <c r="D16" s="15" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
Updates for solving issues and updates for transaction COHV were completed, new version published
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CCDA1352-43BE-4179-B15E-1E2E0669C0D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212667E0-F4FA-4A33-8EE2-3F99807AE43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="114">
   <si>
     <t>Name</t>
   </si>
@@ -382,16 +382,32 @@
   <si>
     <t>C:\Users\aci-cns\Documents\Test UiPath\Informe seguimiento Repuestos\Exceptions_Screenshots</t>
   </si>
+  <si>
+    <t>SplitBatchIntervalZMM026</t>
+  </si>
+  <si>
+    <t>Valor inicial para partir los intervalos de los lotes a la transacción</t>
+  </si>
+  <si>
+    <t>SplitBatchIntervalCOHV</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -508,6 +524,11 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -529,28 +550,32 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -766,7 +791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z997"/>
+  <dimension ref="A1:Z999"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -909,7 +934,7 @@
       </c>
     </row>
     <row r="11" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="A11" s="19" t="s">
         <v>97</v>
       </c>
       <c r="B11" s="14" t="s">
@@ -920,40 +945,60 @@
       </c>
     </row>
     <row r="12" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="16" t="s">
+      <c r="A12" s="19" t="s">
+        <v>111</v>
+      </c>
+      <c r="B12" s="20">
+        <v>35002000</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A13" s="19" t="s">
+        <v>113</v>
+      </c>
+      <c r="B13" s="20">
+        <v>35002000</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="16" t="s">
         <v>101</v>
       </c>
-      <c r="B12" s="17" t="s">
+      <c r="B14" s="17" t="s">
         <v>102</v>
       </c>
-      <c r="C12" s="5" t="s">
+      <c r="C14" s="5" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="13" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="16" t="s">
+    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="16" t="s">
+      <c r="B15" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="18" t="s">
+    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="B14" s="18" t="s">
+      <c r="B16" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1155,8 +1200,8 @@
     <row r="215" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="216" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="218" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="219" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1935,7 +1980,10 @@
     <row r="995" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="996" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
+  <phoneticPr fontId="19" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Updates for solving delays issue for transaction ZPP029_1 were completed
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{212667E0-F4FA-4A33-8EE2-3F99807AE43B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F87597-2912-4FC7-BE79-519B7D459F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="115">
   <si>
     <t>Name</t>
   </si>
@@ -391,16 +391,26 @@
   <si>
     <t>SplitBatchIntervalCOHV</t>
   </si>
+  <si>
+    <t>SplitBatchIntervalZPP029_1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="21" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -550,32 +560,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -791,7 +802,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:Z999"/>
+  <dimension ref="A1:Z1000"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="43.5703125" customWidth="1"/>
@@ -967,54 +978,64 @@
       </c>
     </row>
     <row r="14" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="16" t="s">
-        <v>101</v>
-      </c>
-      <c r="B14" s="17" t="s">
-        <v>102</v>
+      <c r="A14" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="B14" s="20">
+        <v>35002000</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="16" t="s">
+        <v>101</v>
+      </c>
+      <c r="B15" s="17" t="s">
+        <v>102</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="16" t="s">
         <v>103</v>
       </c>
-      <c r="B15" s="16" t="s">
+      <c r="B16" s="16" t="s">
         <v>104</v>
       </c>
-      <c r="C15" s="5" t="s">
+      <c r="C16" s="5" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="16" spans="1:26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="18" t="s">
+    <row r="17" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="18" t="s">
         <v>107</v>
       </c>
-      <c r="B16" s="18" t="s">
+      <c r="B17" s="18" t="s">
         <v>108</v>
       </c>
-      <c r="C16" s="5" t="s">
+      <c r="C17" s="5" t="s">
         <v>109</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1202,7 +1223,7 @@
     <row r="217" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="218" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="219" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="220" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="220" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="221" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="222" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="223" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1982,8 +2003,9 @@
     <row r="997" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="998" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="19" type="noConversion"/>
+  <phoneticPr fontId="20" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
Update for the ODM repor was completed
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5F87597-2912-4FC7-BE79-519B7D459F47}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C02D0CAE-B3A5-4AA4-AAE5-4A9BB97B519A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="118">
   <si>
     <t>Name</t>
   </si>
@@ -394,16 +394,32 @@
   <si>
     <t>SplitBatchIntervalZPP029_1</t>
   </si>
+  <si>
+    <t>ISR_OnDemandData</t>
+  </si>
+  <si>
+    <t>Asset usado para ejecutar el proceso OnDemand</t>
+  </si>
+  <si>
+    <t>OnDemandData</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="22" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -560,31 +576,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left"/>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
@@ -2005,7 +2025,7 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="20" type="noConversion"/>
+  <phoneticPr fontId="21" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3437,22 +3457,35 @@
         <v>100</v>
       </c>
     </row>
-    <row r="17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="18" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="22" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="23" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="24" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="25" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="26" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="27" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="17" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="23" t="s">
+        <v>117</v>
+      </c>
+      <c r="B17" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D17" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="18" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="19" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="20" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="21" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="22" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="25" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="26" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="27" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="28" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="29" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="30" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="31" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="32" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="33" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="34" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="35" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>

<commit_message>
OnDemand updates and notification by error without macro completed were completed
</commit_message>
<xml_diff>
--- a/Data/Config.xlsx
+++ b/Data/Config.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aci-cns\Documents\UiPath\AMP06_00_InformeSeguimientoRepuestos\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C02D0CAE-B3A5-4AA4-AAE5-4A9BB97B519A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CC7C52D-E856-4D40-A644-1551FC7A3C23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="118">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="166" uniqueCount="130">
   <si>
     <t>Name</t>
   </si>
@@ -403,16 +403,66 @@
   <si>
     <t>OnDemandData</t>
   </si>
+  <si>
+    <t>OnDemandData_Set</t>
+  </si>
+  <si>
+    <t>PosiSoftEmailSender</t>
+  </si>
+  <si>
+    <t>SmtpEmailserver</t>
+  </si>
+  <si>
+    <t>smtp.office365.com</t>
+  </si>
+  <si>
+    <t>SmtpPort</t>
+  </si>
+  <si>
+    <t>EmailSender</t>
+  </si>
+  <si>
+    <t>Cuenta para enviar emails</t>
+  </si>
+  <si>
+    <t>Servidor para enviar emails via SMTP</t>
+  </si>
+  <si>
+    <t>Puerto para enviar emails via SMTP</t>
+  </si>
+  <si>
+    <t>RepuestosEmailTo</t>
+  </si>
+  <si>
+    <t>Correos a notificar por errores presentados</t>
+  </si>
+  <si>
+    <t>ISR_RepuestosEmailTo</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="22" x14ac:knownFonts="1">
+  <fonts count="24" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -576,36 +626,38 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -1041,10 +1093,50 @@
         <v>109</v>
       </c>
     </row>
-    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="24" t="s">
+        <v>118</v>
+      </c>
+      <c r="B18" s="22" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="23" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="5" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>120</v>
+      </c>
+      <c r="B20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>122</v>
+      </c>
+      <c r="B21">
+        <v>587</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>126</v>
+      </c>
+    </row>
     <row r="22" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="23" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="24" spans="1:3" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2025,7 +2117,7 @@
     <row r="999" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <phoneticPr fontId="21" type="noConversion"/>
+  <phoneticPr fontId="23" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0" footer="0"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -3458,7 +3550,7 @@
       </c>
     </row>
     <row r="17" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="23" t="s">
+      <c r="A17" s="24" t="s">
         <v>117</v>
       </c>
       <c r="B17" s="22" t="s">
@@ -3471,7 +3563,20 @@
         <v>116</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="18" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="25" t="s">
+        <v>127</v>
+      </c>
+      <c r="B18" s="25" t="s">
+        <v>129</v>
+      </c>
+      <c r="C18" s="10" t="s">
+        <v>7</v>
+      </c>
+      <c r="D18" s="25" t="s">
+        <v>128</v>
+      </c>
+    </row>
     <row r="19" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="20" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="21" spans="1:4" ht="14.25" customHeight="1" x14ac:dyDescent="0.25"/>

</xml_diff>